<commit_message>
feat: add chief accounting, cash receipts and compact ordering for staging
</commit_message>
<xml_diff>
--- a/frontend/public/templates/member-import.xlsx
+++ b/frontend/public/templates/member-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メンバー追加" sheetId="1" r:id="Rfd289e7698114762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rf05e61704c6d4eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メンバー追加" sheetId="1" r:id="R03ad8d4c779749aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rd7c4638b4cb74261"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'メンバー追加'!$A$1:$D$101</x:definedName>
@@ -1007,8 +1007,8 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="D2:D101" allowBlank="1" showInputMessage="1" showErrorMessage="1" showDropDown="0" errorStyle="stop" errorTitle="権限を選択してください" error="一般参加者または担当者を選んでください。" promptTitle="権限" prompt="一般参加者または担当者を選んでください。">
-      <x:formula1>"一般参加者,担当者"</x:formula1>
+    <x:dataValidation type="list" sqref="D2:D101" allowBlank="1" showInputMessage="1" showErrorMessage="1" showDropDown="0" errorStyle="stop" errorTitle="権限を選択してください" error="一般参加者、担当者、主任から選んでください。" promptTitle="権限" prompt="一般参加者、担当者、主任から選んでください。">
+      <x:formula1>"一般参加者,担当者,主任"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C101" allowBlank="1" showInputMessage="1" showErrorMessage="1" showDropDown="0" errorStyle="stop" errorTitle="グループを選択してください" error="クラシック席またはニュークラシック席を選んでください。" promptTitle="グループ" prompt="クラシック席またはニュークラシック席を選んでください。">
       <x:formula1>"クラシック席,ニュークラシック席"</x:formula1>
@@ -1018,7 +1018,7 @@
   <x:pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <x:pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16cbf9246ee54643"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4568bba1cd8449cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1121,12 +1121,13 @@
         <x:v>セルの選択肢から「クラシック席」または「ニュークラシック席」を選びます。席が決まってから入力してください。</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="39" customHeight="1">
+    <x:row r="14" ht="47" customHeight="1">
       <x:c r="A14" s="18" t="str">
         <x:v>権限</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>セルの選択肢から「一般参加者」または「担当者」を選びます。管理者はこのリストから登録できません。</x:v>
+        <x:v>「一般参加者」「担当者」「主任」から選びます。
+主任は全グループの会計を閲覧できます。管理者はこのリストから登録できません。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">

</xml_diff>